<commit_message>
Added Sprint protocol 4 and updated TeamProtokoll
</commit_message>
<xml_diff>
--- a/Sprint_Review_Protocol_4.xlsx
+++ b/Sprint_Review_Protocol_4.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30105"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30110"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\florian\Desktop\itp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{408048EE-66C7-4AED-927C-F815DD9210B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D6933298-C795-43A1-A253-A5A13FE9C9D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{5C77D34F-34C3-4D2F-849C-09193AE86D67}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="104">
   <si>
     <t>Sprint Review Protocol</t>
   </si>
@@ -143,6 +143,141 @@
     <t>Durch Vorerfahrung war die Umsetzung relativ einfach</t>
   </si>
   <si>
+    <t>S4AD1</t>
+  </si>
+  <si>
+    <t>Ambient Sounds</t>
+  </si>
+  <si>
+    <t>Alles ging gut wenige Probleme und Fehler</t>
+  </si>
+  <si>
+    <t>S4AD2</t>
+  </si>
+  <si>
+    <t>Enemy Chase Sound</t>
+  </si>
+  <si>
+    <t>Probleme bei der Implementation</t>
+  </si>
+  <si>
+    <t>S4AD3</t>
+  </si>
+  <si>
+    <t>Enemy Steps</t>
+  </si>
+  <si>
+    <t>Implementation anfangs schwieriger als gedacht, jedoch alles gut geschafft</t>
+  </si>
+  <si>
+    <t>S4SH1</t>
+  </si>
+  <si>
+    <t>Eingangshalle</t>
+  </si>
+  <si>
+    <t>Kleine Platzierungsfehler, mussten nochmal überarbeitet werden</t>
+  </si>
+  <si>
+    <t>S4SH2</t>
+  </si>
+  <si>
+    <t>Turnsaal</t>
+  </si>
+  <si>
+    <t>Erstes mal mit custom materials gearbeitet</t>
+  </si>
+  <si>
+    <t>S4SH3</t>
+  </si>
+  <si>
+    <t>Klassenraum 5</t>
+  </si>
+  <si>
+    <t>Kopie von altem Klassenraum verwendet</t>
+  </si>
+  <si>
+    <t>S4SH4</t>
+  </si>
+  <si>
+    <t>Stockwerk -1</t>
+  </si>
+  <si>
+    <t>Beleuchtung in eigenen Task verschoben</t>
+  </si>
+  <si>
+    <t>S3SH1</t>
+  </si>
+  <si>
+    <t>Aufzugsschaft inkl. Aufzug</t>
+  </si>
+  <si>
+    <t>Aufzug und Kabel noch nicht fertig weil custom assets benötigt werden</t>
+  </si>
+  <si>
+    <t>S4SM1</t>
+  </si>
+  <si>
+    <t>Keycards erstellen</t>
+  </si>
+  <si>
+    <t>Schnellere Implementierung in Unreal als im letzten Sprint</t>
+  </si>
+  <si>
+    <t>S4SM2</t>
+  </si>
+  <si>
+    <t>Objektplatzierung in Räumen</t>
+  </si>
+  <si>
+    <t>Die Räume wurden noch nicht alle erstellt bzw. erst kurz vor Ende erstellt</t>
+  </si>
+  <si>
+    <t>S3SM3</t>
+  </si>
+  <si>
+    <t>Objekte hinzufügen</t>
+  </si>
+  <si>
+    <t>Das Bathroom hat vom letzten Sprint gefehlt</t>
+  </si>
+  <si>
+    <t>S4MS1</t>
+  </si>
+  <si>
+    <t>Animationr/Rigging Pt3</t>
+  </si>
+  <si>
+    <t>Mangelndes Zeitmanagement</t>
+  </si>
+  <si>
+    <t>S4MS2</t>
+  </si>
+  <si>
+    <t>Pathfinding/Collision</t>
+  </si>
+  <si>
+    <t>Funktionen von NavMesh nicht umgesetzt</t>
+  </si>
+  <si>
+    <t>S4MS3</t>
+  </si>
+  <si>
+    <t>Enemy open door logic</t>
+  </si>
+  <si>
+    <t>Implementation schwieriger als gedacht</t>
+  </si>
+  <si>
+    <t>S4MS4</t>
+  </si>
+  <si>
+    <t>Enemy lose sight logic</t>
+  </si>
+  <si>
+    <t>Testing schwierig da Pathfinding Probleme</t>
+  </si>
+  <si>
     <t>Liked</t>
   </si>
   <si>
@@ -153,6 +288,54 @@
   </si>
   <si>
     <t>Longed for</t>
+  </si>
+  <si>
+    <t>Erfolgreiche Implementation der Steps und Ambient-Sounds</t>
+  </si>
+  <si>
+    <t>Wie man neue Klassen erstellt und diese auch implementiert</t>
+  </si>
+  <si>
+    <t>Fehlende Erfahrung im Enemy Blueprint</t>
+  </si>
+  <si>
+    <t>Mehr Zeit für Feintuning und Problemlösung</t>
+  </si>
+  <si>
+    <t>Erzielter Fortschritt</t>
+  </si>
+  <si>
+    <t>Custom Materialien erstellen</t>
+  </si>
+  <si>
+    <t>Kreativität bei umsetzen der Ideen</t>
+  </si>
+  <si>
+    <t>Mehr vorgefertigte Assets für das Projekt</t>
+  </si>
+  <si>
+    <t>Es gefiel mir, ein besseres Verständnis für BP zu erlernen</t>
+  </si>
+  <si>
+    <t>Ich habe gelernt, BP-Objekte miteinander zu verbinden und korrekt in die Spielwelt einzusetzen</t>
+  </si>
+  <si>
+    <t>Es fehlt mir noch an Wissen darüber, wie man Objekte erstellt und wie man mit Nodes arbeitet</t>
+  </si>
+  <si>
+    <t>Mehr Zeit damit zu verbringen, selbst in Unreal Engine Objekte zu erstellen und zu verbinden</t>
+  </si>
+  <si>
+    <t>Animationsanpassaung war einfacher durch Erfahrung der letzten Sprints</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Besseres Verständnis in Unreal Engine5 Blueprints im Bezug auf Pathfinding und AI Movement</t>
+  </si>
+  <si>
+    <t>Besseres Zeitmangement um die geplanten Features in der vorgegebenen Zeit umzusetzen</t>
+  </si>
+  <si>
+    <t>Kenntniss über NavMesh</t>
   </si>
   <si>
     <t>Erfolgreiche Implementation des Card Scanners</t>
@@ -171,7 +354,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -220,6 +403,12 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="6">
@@ -445,9 +634,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -487,6 +673,15 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -505,14 +700,8 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
@@ -849,168 +1038,168 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
-      <c r="I1" s="20"/>
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
+      <c r="G1" s="22"/>
+      <c r="H1" s="22"/>
+      <c r="I1" s="22"/>
     </row>
     <row r="2" spans="1:9">
-      <c r="A2" s="20"/>
-      <c r="B2" s="20"/>
-      <c r="C2" s="20"/>
-      <c r="D2" s="20"/>
-      <c r="E2" s="20"/>
-      <c r="F2" s="20"/>
-      <c r="G2" s="20"/>
-      <c r="H2" s="20"/>
-      <c r="I2" s="20"/>
+      <c r="A2" s="22"/>
+      <c r="B2" s="22"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
+      <c r="G2" s="22"/>
+      <c r="H2" s="22"/>
+      <c r="I2" s="22"/>
     </row>
     <row r="3" spans="1:9" ht="26.25">
-      <c r="A3" s="13"/>
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
-      <c r="E3" s="13"/>
-      <c r="F3" s="13"/>
-      <c r="G3" s="13"/>
-      <c r="H3" s="13"/>
-      <c r="I3" s="13"/>
+      <c r="A3" s="12"/>
+      <c r="B3" s="12"/>
+      <c r="C3" s="12"/>
+      <c r="D3" s="12"/>
+      <c r="E3" s="12"/>
+      <c r="F3" s="12"/>
+      <c r="G3" s="12"/>
+      <c r="H3" s="12"/>
+      <c r="I3" s="12"/>
     </row>
     <row r="4" spans="1:9">
       <c r="A4" s="29" t="s">
         <v>1</v>
       </c>
       <c r="B4" s="30"/>
-      <c r="C4" s="22">
+      <c r="C4" s="24">
         <v>4</v>
       </c>
-      <c r="D4" s="22"/>
-      <c r="E4" s="22"/>
-      <c r="F4" s="22"/>
-      <c r="G4" s="22"/>
+      <c r="D4" s="24"/>
+      <c r="E4" s="24"/>
+      <c r="F4" s="24"/>
+      <c r="G4" s="24"/>
     </row>
     <row r="5" spans="1:9">
       <c r="A5" s="31" t="s">
         <v>2</v>
       </c>
       <c r="B5" s="32"/>
-      <c r="C5" s="23">
+      <c r="C5" s="25">
         <v>46154</v>
       </c>
-      <c r="D5" s="23"/>
-      <c r="E5" s="23"/>
-      <c r="F5" s="23"/>
-      <c r="G5" s="23"/>
+      <c r="D5" s="25"/>
+      <c r="E5" s="25"/>
+      <c r="F5" s="25"/>
+      <c r="G5" s="25"/>
     </row>
     <row r="6" spans="1:9">
       <c r="A6" s="31" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="32"/>
-      <c r="C6" s="24">
+      <c r="C6" s="26">
         <v>35</v>
       </c>
-      <c r="D6" s="24"/>
-      <c r="E6" s="24"/>
-      <c r="F6" s="24"/>
-      <c r="G6" s="24"/>
+      <c r="D6" s="26"/>
+      <c r="E6" s="26"/>
+      <c r="F6" s="26"/>
+      <c r="G6" s="26"/>
     </row>
     <row r="7" spans="1:9">
       <c r="A7" s="31" t="s">
         <v>4</v>
       </c>
       <c r="B7" s="32"/>
-      <c r="C7" s="25" t="s">
+      <c r="C7" s="27" t="s">
         <v>5</v>
       </c>
-      <c r="D7" s="25"/>
-      <c r="E7" s="25"/>
-      <c r="F7" s="25"/>
-      <c r="G7" s="25"/>
+      <c r="D7" s="27"/>
+      <c r="E7" s="27"/>
+      <c r="F7" s="27"/>
+      <c r="G7" s="27"/>
     </row>
     <row r="8" spans="1:9">
       <c r="A8" s="31" t="s">
         <v>6</v>
       </c>
       <c r="B8" s="32"/>
-      <c r="C8" s="21" t="s">
+      <c r="C8" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="D8" s="21"/>
-      <c r="E8" s="21"/>
-      <c r="F8" s="21"/>
-      <c r="G8" s="21"/>
+      <c r="D8" s="23"/>
+      <c r="E8" s="23"/>
+      <c r="F8" s="23"/>
+      <c r="G8" s="23"/>
     </row>
     <row r="9" spans="1:9">
       <c r="A9" s="31" t="s">
         <v>8</v>
       </c>
       <c r="B9" s="32"/>
-      <c r="C9" s="21" t="s">
+      <c r="C9" s="23" t="s">
         <v>9</v>
       </c>
-      <c r="D9" s="21"/>
-      <c r="E9" s="21"/>
-      <c r="F9" s="21"/>
-      <c r="G9" s="21"/>
+      <c r="D9" s="23"/>
+      <c r="E9" s="23"/>
+      <c r="F9" s="23"/>
+      <c r="G9" s="23"/>
     </row>
     <row r="10" spans="1:9">
       <c r="A10" s="31" t="s">
         <v>10</v>
       </c>
       <c r="B10" s="32"/>
-      <c r="C10" s="21" t="s">
+      <c r="C10" s="23" t="s">
         <v>11</v>
       </c>
-      <c r="D10" s="21"/>
-      <c r="E10" s="21"/>
-      <c r="F10" s="21"/>
-      <c r="G10" s="21"/>
+      <c r="D10" s="23"/>
+      <c r="E10" s="23"/>
+      <c r="F10" s="23"/>
+      <c r="G10" s="23"/>
     </row>
     <row r="11" spans="1:9">
       <c r="A11" s="31" t="s">
         <v>12</v>
       </c>
       <c r="B11" s="32"/>
-      <c r="C11" s="28" t="s">
+      <c r="C11" s="21" t="s">
         <v>13</v>
       </c>
-      <c r="D11" s="28"/>
-      <c r="E11" s="28"/>
-      <c r="F11" s="28"/>
-      <c r="G11" s="28"/>
+      <c r="D11" s="21"/>
+      <c r="E11" s="21"/>
+      <c r="F11" s="21"/>
+      <c r="G11" s="21"/>
     </row>
     <row r="12" spans="1:9">
       <c r="A12" s="33" t="s">
         <v>14</v>
       </c>
       <c r="B12" s="34"/>
-      <c r="C12" s="26" t="s">
+      <c r="C12" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="D12" s="26"/>
-      <c r="E12" s="26"/>
-      <c r="F12" s="26"/>
-      <c r="G12" s="26"/>
+      <c r="D12" s="19"/>
+      <c r="E12" s="19"/>
+      <c r="F12" s="19"/>
+      <c r="G12" s="19"/>
     </row>
     <row r="14" spans="1:9">
-      <c r="A14" s="27" t="s">
+      <c r="A14" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="B14" s="27"/>
-      <c r="C14" s="27"/>
-      <c r="D14" s="27"/>
-      <c r="E14" s="27"/>
-      <c r="F14" s="27"/>
-      <c r="G14" s="27"/>
-      <c r="H14" s="27"/>
+      <c r="B14" s="20"/>
+      <c r="C14" s="20"/>
+      <c r="D14" s="20"/>
+      <c r="E14" s="20"/>
+      <c r="F14" s="20"/>
+      <c r="G14" s="20"/>
+      <c r="H14" s="20"/>
     </row>
     <row r="15" spans="1:9">
       <c r="A15" s="1" t="s">
@@ -1039,274 +1228,454 @@
       </c>
     </row>
     <row r="16" spans="1:9" ht="50.25" customHeight="1">
-      <c r="A16" s="16" t="s">
+      <c r="A16" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="B16" s="16" t="s">
+      <c r="B16" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="C16" s="16">
+      <c r="C16" s="15">
         <v>2</v>
       </c>
-      <c r="D16" s="16">
+      <c r="D16" s="15">
         <v>4</v>
       </c>
       <c r="E16" s="5">
         <f>D16-C16</f>
         <v>2</v>
       </c>
-      <c r="F16" s="14" t="s">
+      <c r="F16" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="G16" s="15"/>
-      <c r="H16" s="17" t="s">
+      <c r="G16" s="14"/>
+      <c r="H16" s="16" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="50.25" customHeight="1">
-      <c r="A17" s="16" t="s">
+      <c r="A17" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="B17" s="16" t="s">
+      <c r="B17" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="C17" s="16">
+      <c r="C17" s="15">
         <v>1</v>
       </c>
-      <c r="D17" s="16">
+      <c r="D17" s="15">
         <v>1</v>
       </c>
       <c r="E17" s="5">
         <f t="shared" ref="E17:E33" si="0">D17-C17</f>
         <v>0</v>
       </c>
-      <c r="F17" s="14" t="s">
+      <c r="F17" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="G17" s="15"/>
-      <c r="H17" s="17" t="s">
+      <c r="G17" s="14"/>
+      <c r="H17" s="16" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="50.25" customHeight="1">
-      <c r="A18" s="16" t="s">
+      <c r="A18" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="B18" s="16" t="s">
+      <c r="B18" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="C18" s="16">
+      <c r="C18" s="15">
         <v>1</v>
       </c>
-      <c r="D18" s="16">
+      <c r="D18" s="15">
         <v>0.5</v>
       </c>
       <c r="E18" s="5">
         <f t="shared" si="0"/>
         <v>-0.5</v>
       </c>
-      <c r="F18" s="14" t="s">
+      <c r="F18" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="G18" s="15"/>
-      <c r="H18" s="17" t="s">
+      <c r="G18" s="14"/>
+      <c r="H18" s="16" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="50.25" customHeight="1">
-      <c r="A19" s="16"/>
-      <c r="B19" s="16"/>
-      <c r="C19" s="16"/>
-      <c r="D19" s="16"/>
+      <c r="A19" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="B19" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="C19" s="15">
+        <v>5</v>
+      </c>
+      <c r="D19" s="15">
+        <v>4</v>
+      </c>
       <c r="E19" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="F19" s="14"/>
-      <c r="G19" s="15"/>
-      <c r="H19" s="17"/>
+        <v>-1</v>
+      </c>
+      <c r="F19" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="G19" s="14"/>
+      <c r="H19" s="16" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="20" spans="1:8" ht="50.25" customHeight="1">
-      <c r="A20" s="16"/>
-      <c r="B20" s="17"/>
-      <c r="C20" s="16"/>
-      <c r="D20" s="16"/>
+      <c r="A20" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="C20" s="15">
+        <v>2</v>
+      </c>
+      <c r="D20" s="15">
+        <v>3</v>
+      </c>
       <c r="E20" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="F20" s="14"/>
-      <c r="G20" s="15"/>
-      <c r="H20" s="17"/>
+        <v>1</v>
+      </c>
+      <c r="F20" s="13"/>
+      <c r="G20" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="H20" s="16" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="21" spans="1:8" ht="50.25" customHeight="1">
-      <c r="A21" s="16"/>
-      <c r="B21" s="16"/>
-      <c r="C21" s="16"/>
-      <c r="D21" s="16"/>
+      <c r="A21" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="B21" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="C21" s="15">
+        <v>3</v>
+      </c>
+      <c r="D21" s="15">
+        <v>3</v>
+      </c>
       <c r="E21" s="5">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F21" s="14"/>
-      <c r="G21" s="15"/>
-      <c r="H21" s="17"/>
+      <c r="F21" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="G21" s="14"/>
+      <c r="H21" s="16" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="22" spans="1:8" ht="50.25" customHeight="1">
-      <c r="A22" s="16"/>
-      <c r="B22" s="16"/>
-      <c r="C22" s="16"/>
-      <c r="D22" s="16"/>
+      <c r="A22" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="B22" s="15" t="s">
+        <v>45</v>
+      </c>
+      <c r="C22" s="15">
+        <v>4</v>
+      </c>
+      <c r="D22" s="15">
+        <v>3</v>
+      </c>
       <c r="E22" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="F22" s="14"/>
-      <c r="G22" s="15"/>
-      <c r="H22" s="17"/>
+        <v>-1</v>
+      </c>
+      <c r="F22" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="G22" s="14"/>
+      <c r="H22" s="16" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="23" spans="1:8" ht="50.25" customHeight="1">
-      <c r="A23" s="16"/>
-      <c r="B23" s="16"/>
-      <c r="C23" s="16"/>
-      <c r="D23" s="16"/>
+      <c r="A23" s="15" t="s">
+        <v>47</v>
+      </c>
+      <c r="B23" s="15" t="s">
+        <v>48</v>
+      </c>
+      <c r="C23" s="15">
+        <v>3</v>
+      </c>
+      <c r="D23" s="15">
+        <v>3</v>
+      </c>
       <c r="E23" s="5">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F23" s="14"/>
-      <c r="G23" s="15"/>
-      <c r="H23" s="17"/>
+      <c r="F23" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="G23" s="14"/>
+      <c r="H23" s="16" t="s">
+        <v>49</v>
+      </c>
     </row>
     <row r="24" spans="1:8" ht="50.25" customHeight="1">
-      <c r="A24" s="16"/>
-      <c r="B24" s="16"/>
-      <c r="C24" s="16"/>
-      <c r="D24" s="16"/>
+      <c r="A24" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="B24" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="C24" s="15">
+        <v>0.5</v>
+      </c>
+      <c r="D24" s="15">
+        <v>0.5</v>
+      </c>
       <c r="E24" s="5">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F24" s="14"/>
-      <c r="G24" s="15"/>
-      <c r="H24" s="16"/>
+      <c r="F24" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="G24" s="14"/>
+      <c r="H24" s="16" t="s">
+        <v>52</v>
+      </c>
     </row>
     <row r="25" spans="1:8" ht="50.25" customHeight="1">
-      <c r="A25" s="16"/>
-      <c r="B25" s="16"/>
-      <c r="C25" s="16"/>
-      <c r="D25" s="16"/>
+      <c r="A25" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="B25" s="15" t="s">
+        <v>54</v>
+      </c>
+      <c r="C25" s="15">
+        <v>3</v>
+      </c>
+      <c r="D25" s="15">
+        <v>2</v>
+      </c>
       <c r="E25" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="F25" s="14"/>
-      <c r="G25" s="15"/>
-      <c r="H25" s="17"/>
+        <v>-1</v>
+      </c>
+      <c r="F25" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="G25" s="14"/>
+      <c r="H25" s="16" t="s">
+        <v>55</v>
+      </c>
     </row>
     <row r="26" spans="1:8" ht="50.25" customHeight="1">
-      <c r="A26" s="16"/>
-      <c r="B26" s="16"/>
-      <c r="C26" s="16"/>
-      <c r="D26" s="16"/>
+      <c r="A26" s="15" t="s">
+        <v>56</v>
+      </c>
+      <c r="B26" s="15" t="s">
+        <v>57</v>
+      </c>
+      <c r="C26" s="15">
+        <v>4</v>
+      </c>
+      <c r="D26" s="15">
+        <v>3</v>
+      </c>
       <c r="E26" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="F26" s="14"/>
-      <c r="G26" s="15"/>
-      <c r="H26" s="16"/>
+        <v>-1</v>
+      </c>
+      <c r="F26" s="13"/>
+      <c r="G26" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="H26" s="16" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="27" spans="1:8" ht="50.25" customHeight="1">
-      <c r="A27" s="16"/>
-      <c r="B27" s="16"/>
-      <c r="C27" s="16"/>
-      <c r="D27" s="16"/>
+      <c r="A27" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="B27" s="15" t="s">
+        <v>60</v>
+      </c>
+      <c r="C27" s="15">
+        <v>2</v>
+      </c>
+      <c r="D27" s="15">
+        <v>3</v>
+      </c>
       <c r="E27" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="F27" s="14"/>
-      <c r="G27" s="15"/>
-      <c r="H27" s="17"/>
+        <v>1</v>
+      </c>
+      <c r="F27" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="G27" s="14"/>
+      <c r="H27" s="16" t="s">
+        <v>61</v>
+      </c>
     </row>
     <row r="28" spans="1:8" ht="50.25" customHeight="1">
-      <c r="A28" s="16"/>
-      <c r="B28" s="16"/>
-      <c r="C28" s="16"/>
-      <c r="D28" s="16"/>
+      <c r="A28" s="15" t="s">
+        <v>62</v>
+      </c>
+      <c r="B28" s="15" t="s">
+        <v>63</v>
+      </c>
+      <c r="C28" s="15">
+        <v>3</v>
+      </c>
+      <c r="D28" s="15">
+        <v>4</v>
+      </c>
       <c r="E28" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="F28" s="14"/>
-      <c r="G28" s="15"/>
-      <c r="H28" s="16"/>
+        <v>1</v>
+      </c>
+      <c r="F28" s="13"/>
+      <c r="G28" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="H28" s="16" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="29" spans="1:8" ht="50.25" customHeight="1">
-      <c r="A29" s="16"/>
-      <c r="B29" s="16"/>
-      <c r="C29" s="16"/>
-      <c r="D29" s="16"/>
+      <c r="A29" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="B29" s="15" t="s">
+        <v>66</v>
+      </c>
+      <c r="C29" s="15">
+        <v>4</v>
+      </c>
+      <c r="D29" s="15">
+        <v>5</v>
+      </c>
       <c r="E29" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="F29" s="14"/>
-      <c r="G29" s="15"/>
-      <c r="H29" s="16"/>
+        <v>1</v>
+      </c>
+      <c r="F29" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="G29" s="14"/>
+      <c r="H29" s="16" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="30" spans="1:8" ht="50.25" customHeight="1">
-      <c r="A30" s="16"/>
-      <c r="B30" s="16"/>
-      <c r="C30" s="16"/>
-      <c r="D30" s="16"/>
+      <c r="A30" s="15" t="s">
+        <v>68</v>
+      </c>
+      <c r="B30" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="C30" s="15">
+        <v>1.5</v>
+      </c>
+      <c r="D30" s="15">
+        <v>0.5</v>
+      </c>
       <c r="E30" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="F30" s="14"/>
-      <c r="G30" s="15"/>
-      <c r="H30" s="17"/>
+        <v>-1</v>
+      </c>
+      <c r="F30" s="13"/>
+      <c r="G30" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="H30" s="16" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="31" spans="1:8" ht="50.25" customHeight="1">
-      <c r="A31" s="16"/>
-      <c r="B31" s="16"/>
-      <c r="C31" s="16"/>
-      <c r="D31" s="16"/>
+      <c r="A31" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="B31" s="15" t="s">
+        <v>72</v>
+      </c>
+      <c r="C31" s="15">
+        <v>2</v>
+      </c>
+      <c r="D31" s="15">
+        <v>2.5</v>
+      </c>
       <c r="E31" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="F31" s="14"/>
-      <c r="G31" s="15"/>
-      <c r="H31" s="17"/>
+        <v>0.5</v>
+      </c>
+      <c r="F31" s="13"/>
+      <c r="G31" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="H31" s="16" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="32" spans="1:8" ht="50.25" customHeight="1">
-      <c r="A32" s="16"/>
-      <c r="B32" s="16"/>
-      <c r="C32" s="16"/>
-      <c r="D32" s="16"/>
+      <c r="A32" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="B32" s="15" t="s">
+        <v>75</v>
+      </c>
+      <c r="C32" s="15">
+        <v>1</v>
+      </c>
+      <c r="D32" s="15">
+        <v>1</v>
+      </c>
       <c r="E32" s="5">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F32" s="14"/>
-      <c r="G32" s="15"/>
-      <c r="H32" s="17"/>
+      <c r="F32" s="13"/>
+      <c r="G32" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="H32" s="16" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="33" spans="1:8" ht="50.25" customHeight="1">
-      <c r="A33" s="16"/>
-      <c r="B33" s="16"/>
-      <c r="C33" s="16"/>
-      <c r="D33" s="16"/>
+      <c r="A33" s="15" t="s">
+        <v>77</v>
+      </c>
+      <c r="B33" s="15" t="s">
+        <v>78</v>
+      </c>
+      <c r="C33" s="15">
+        <v>1.5</v>
+      </c>
+      <c r="D33" s="15">
+        <v>2</v>
+      </c>
       <c r="E33" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="F33" s="14"/>
-      <c r="G33" s="15"/>
-      <c r="H33" s="16"/>
+        <v>0.5</v>
+      </c>
+      <c r="F33" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="G33" s="14"/>
+      <c r="H33" s="16" t="s">
+        <v>79</v>
+      </c>
     </row>
     <row r="34" spans="1:8">
       <c r="A34" s="3">
@@ -1318,7 +1687,7 @@
       <c r="D34" s="3"/>
       <c r="E34" s="3">
         <f>SUM(E16:E25)</f>
-        <v>1.5</v>
+        <v>-0.5</v>
       </c>
       <c r="F34" s="3">
         <f>COUNT(F16:F25)</f>
@@ -1332,81 +1701,107 @@
     </row>
     <row r="36" spans="1:8" ht="24.75" customHeight="1">
       <c r="B36" s="4"/>
-      <c r="C36" s="10" t="s">
-        <v>35</v>
-      </c>
-      <c r="D36" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="E36" s="10" t="s">
-        <v>37</v>
-      </c>
-      <c r="F36" s="11" t="s">
-        <v>38</v>
+      <c r="C36" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="D36" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="E36" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="F36" s="10" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="37" spans="1:8" ht="60" customHeight="1">
-      <c r="B37" s="8" t="s">
+      <c r="B37" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="C37" s="18"/>
-      <c r="D37" s="18"/>
-      <c r="E37" s="18"/>
-      <c r="F37" s="6"/>
-    </row>
-    <row r="38" spans="1:8" ht="60" customHeight="1">
+      <c r="C37" s="17" t="s">
+        <v>84</v>
+      </c>
+      <c r="D37" s="17" t="s">
+        <v>85</v>
+      </c>
+      <c r="E37" s="17" t="s">
+        <v>86</v>
+      </c>
+      <c r="F37" s="18" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" ht="53.25" customHeight="1">
       <c r="A38"/>
-      <c r="B38" s="8" t="s">
+      <c r="B38" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="C38" s="18"/>
-      <c r="D38" s="18"/>
-      <c r="E38" s="5"/>
-      <c r="F38" s="19"/>
-    </row>
-    <row r="39" spans="1:8" ht="60" customHeight="1">
-      <c r="B39" s="8" t="s">
+      <c r="C38" s="17" t="s">
+        <v>88</v>
+      </c>
+      <c r="D38" s="17" t="s">
+        <v>89</v>
+      </c>
+      <c r="E38" s="17" t="s">
+        <v>90</v>
+      </c>
+      <c r="F38" s="18" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" ht="96" customHeight="1">
+      <c r="B39" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="C39" s="18"/>
-      <c r="D39" s="5"/>
-      <c r="E39" s="18"/>
-      <c r="F39" s="19"/>
-    </row>
-    <row r="40" spans="1:8" ht="60" customHeight="1">
-      <c r="B40" s="8" t="s">
+      <c r="C39" s="17" t="s">
+        <v>92</v>
+      </c>
+      <c r="D39" s="17" t="s">
+        <v>93</v>
+      </c>
+      <c r="E39" s="17" t="s">
+        <v>94</v>
+      </c>
+      <c r="F39" s="18" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" ht="90.75" customHeight="1">
+      <c r="B40" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C40" s="18"/>
-      <c r="D40" s="18"/>
-      <c r="E40" s="18"/>
-      <c r="F40" s="19"/>
+      <c r="C40" s="17" t="s">
+        <v>96</v>
+      </c>
+      <c r="D40" s="17" t="s">
+        <v>97</v>
+      </c>
+      <c r="E40" s="17" t="s">
+        <v>98</v>
+      </c>
+      <c r="F40" s="28" t="s">
+        <v>99</v>
+      </c>
     </row>
     <row r="41" spans="1:8" ht="60" customHeight="1">
-      <c r="B41" s="9" t="s">
+      <c r="B41" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="C41" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="D41" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="E41" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="F41" s="12" t="s">
-        <v>42</v>
+      <c r="C41" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="D41" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="E41" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="F41" s="11" t="s">
+        <v>103</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="20">
-    <mergeCell ref="C12:G12"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="A11:B11"/>
-    <mergeCell ref="A12:B12"/>
-    <mergeCell ref="A14:H14"/>
-    <mergeCell ref="C11:G11"/>
     <mergeCell ref="A1:I2"/>
     <mergeCell ref="C9:G9"/>
     <mergeCell ref="C10:G10"/>
@@ -1421,6 +1816,12 @@
     <mergeCell ref="C6:G6"/>
     <mergeCell ref="C7:G7"/>
     <mergeCell ref="C8:G8"/>
+    <mergeCell ref="C12:G12"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="A14:H14"/>
+    <mergeCell ref="C11:G11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="60" fitToWidth="0" fitToHeight="0" orientation="landscape" r:id="rId1"/>

</xml_diff>